<commit_message>
Changed game parameters a little
</commit_message>
<xml_diff>
--- a/Docs/UnitsParametersCalculations.xlsx
+++ b/Docs/UnitsParametersCalculations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\REPOS\Rust\FinalRustProject\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E76B1F7-987C-4AC9-94B3-FC22E3ACE9DE}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE5E1C7-DB14-4AAF-9156-579A73629A2E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="3075" windowWidth="22380" windowHeight="11535" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>Health</t>
   </si>
@@ -205,6 +205,12 @@
   </si>
   <si>
     <t>We are summarizing the probabilities, randomizing within this big range and evaluating who's target</t>
+  </si>
+  <si>
+    <t>Abomination</t>
+  </si>
+  <si>
+    <t>Witch</t>
   </si>
 </sst>
 </file>
@@ -517,7 +523,7 @@
       <font>
         <color rgb="FFFFFF00"/>
       </font>
-      <numFmt numFmtId="166" formatCode="0;[Red]0"/>
+      <numFmt numFmtId="164" formatCode="0;[Red]0"/>
       <fill>
         <patternFill>
           <bgColor rgb="FFFF0000"/>
@@ -888,7 +894,7 @@
     </row>
     <row r="5" spans="1:24" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="B5" s="9">
         <v>3</v>
@@ -1237,7 +1243,7 @@
     </row>
     <row r="17" spans="1:18" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="B17" s="9">
         <v>9</v>

</xml_diff>